<commit_message>
fix: prevent management review header clipping
</commit_message>
<xml_diff>
--- a/model/Palmetto_Stay_FP&A_Model.xlsx
+++ b/model/Palmetto_Stay_FP&A_Model.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CAF49B9-7C08-45A6-A294-EA759D0F1271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81052083-78CD-405D-9DCD-1482D85B4399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="2205" windowWidth="15390" windowHeight="9443" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4205,8 +4205,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -4214,17 +4214,23 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="18" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -4307,30 +4313,6 @@
     <xf numFmtId="0" fontId="25" fillId="19" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="16" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="30" fillId="16" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="25" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="19" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="30" fillId="19" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="25" fillId="19" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="20" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -4385,11 +4367,29 @@
     <xf numFmtId="0" fontId="25" fillId="21" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="178" fontId="25" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="178" fontId="25" fillId="19" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="19" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="30" fillId="19" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="30" fillId="16" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -24092,16 +24092,16 @@
       <c r="N21" s="98"/>
     </row>
     <row r="22" spans="3:14" ht="28.05" customHeight="1">
-      <c r="C22" s="261" t="s">
+      <c r="C22" s="258" t="s">
         <v>309</v>
       </c>
-      <c r="D22" s="261"/>
-      <c r="E22" s="261"/>
-      <c r="F22" s="261"/>
-      <c r="G22" s="261"/>
-      <c r="H22" s="261"/>
-      <c r="I22" s="261"/>
-      <c r="J22" s="261"/>
+      <c r="D22" s="258"/>
+      <c r="E22" s="258"/>
+      <c r="F22" s="258"/>
+      <c r="G22" s="258"/>
+      <c r="H22" s="258"/>
+      <c r="I22" s="258"/>
+      <c r="J22" s="258"/>
       <c r="K22" s="98"/>
       <c r="L22" s="98"/>
       <c r="M22" s="98"/>
@@ -25283,16 +25283,16 @@
       <c r="N57" s="98"/>
     </row>
     <row r="58" spans="3:14" ht="28.05" customHeight="1">
-      <c r="C58" s="261" t="s">
+      <c r="C58" s="258" t="s">
         <v>325</v>
       </c>
-      <c r="D58" s="261"/>
-      <c r="E58" s="261"/>
-      <c r="F58" s="261"/>
-      <c r="G58" s="261"/>
-      <c r="H58" s="261"/>
-      <c r="I58" s="261"/>
-      <c r="J58" s="261"/>
+      <c r="D58" s="258"/>
+      <c r="E58" s="258"/>
+      <c r="F58" s="258"/>
+      <c r="G58" s="258"/>
+      <c r="H58" s="258"/>
+      <c r="I58" s="258"/>
+      <c r="J58" s="258"/>
       <c r="K58" s="98"/>
       <c r="L58" s="98"/>
       <c r="M58" s="98"/>
@@ -31903,10 +31903,10 @@
       <c r="D262" s="151" t="s">
         <v>424</v>
       </c>
-      <c r="E262" s="258" t="s">
+      <c r="E262" s="261" t="s">
         <v>425</v>
       </c>
-      <c r="F262" s="258"/>
+      <c r="F262" s="261"/>
       <c r="G262" s="152">
         <f>SUM(F169:G169)</f>
         <v>-37445.039999999994</v>
@@ -31914,10 +31914,10 @@
       <c r="H262" s="151" t="s">
         <v>426</v>
       </c>
-      <c r="I262" s="258" t="s">
+      <c r="I262" s="261" t="s">
         <v>427</v>
       </c>
-      <c r="J262" s="258"/>
+      <c r="J262" s="261"/>
       <c r="K262" s="151" t="s">
         <v>95</v>
       </c>
@@ -31938,10 +31938,10 @@
       <c r="D263" s="151" t="s">
         <v>432</v>
       </c>
-      <c r="E263" s="258" t="s">
+      <c r="E263" s="261" t="s">
         <v>433</v>
       </c>
-      <c r="F263" s="258"/>
+      <c r="F263" s="261"/>
       <c r="G263" s="152">
         <f>J170</f>
         <v>-17667.04999999989</v>
@@ -31949,10 +31949,10 @@
       <c r="H263" s="151" t="s">
         <v>194</v>
       </c>
-      <c r="I263" s="258" t="s">
+      <c r="I263" s="261" t="s">
         <v>434</v>
       </c>
-      <c r="J263" s="258"/>
+      <c r="J263" s="261"/>
       <c r="K263" s="151" t="s">
         <v>95</v>
       </c>
@@ -31973,10 +31973,10 @@
       <c r="D264" s="151" t="s">
         <v>439</v>
       </c>
-      <c r="E264" s="258" t="s">
+      <c r="E264" s="261" t="s">
         <v>440</v>
       </c>
-      <c r="F264" s="258"/>
+      <c r="F264" s="261"/>
       <c r="G264" s="152">
         <f>SUM(G191:I191)</f>
         <v>4700.9999999999909</v>
@@ -31984,10 +31984,10 @@
       <c r="H264" s="151" t="s">
         <v>441</v>
       </c>
-      <c r="I264" s="258" t="s">
+      <c r="I264" s="261" t="s">
         <v>442</v>
       </c>
-      <c r="J264" s="258"/>
+      <c r="J264" s="261"/>
       <c r="K264" s="151" t="s">
         <v>95</v>
       </c>
@@ -32008,10 +32008,10 @@
       <c r="D265" s="151" t="s">
         <v>447</v>
       </c>
-      <c r="E265" s="258" t="s">
+      <c r="E265" s="261" t="s">
         <v>448</v>
       </c>
-      <c r="F265" s="258"/>
+      <c r="F265" s="261"/>
       <c r="G265" s="152">
         <f>SUM(G190:H190)</f>
         <v>7625.6400000000012</v>
@@ -32019,10 +32019,10 @@
       <c r="H265" s="151" t="s">
         <v>449</v>
       </c>
-      <c r="I265" s="258" t="s">
+      <c r="I265" s="261" t="s">
         <v>450</v>
       </c>
-      <c r="J265" s="258"/>
+      <c r="J265" s="261"/>
       <c r="K265" s="151" t="s">
         <v>108</v>
       </c>
@@ -32043,10 +32043,10 @@
       <c r="D266" s="151" t="s">
         <v>455</v>
       </c>
-      <c r="E266" s="258" t="s">
+      <c r="E266" s="261" t="s">
         <v>456</v>
       </c>
-      <c r="F266" s="258"/>
+      <c r="F266" s="261"/>
       <c r="G266" s="152">
         <f>I231</f>
         <v>-18000</v>
@@ -32054,10 +32054,10 @@
       <c r="H266" s="151" t="s">
         <v>457</v>
       </c>
-      <c r="I266" s="258" t="s">
+      <c r="I266" s="261" t="s">
         <v>458</v>
       </c>
-      <c r="J266" s="258"/>
+      <c r="J266" s="261"/>
       <c r="K266" s="151" t="s">
         <v>95</v>
       </c>
@@ -32078,10 +32078,10 @@
       <c r="D267" s="151" t="s">
         <v>463</v>
       </c>
-      <c r="E267" s="258" t="s">
+      <c r="E267" s="261" t="s">
         <v>464</v>
       </c>
-      <c r="F267" s="258"/>
+      <c r="F267" s="261"/>
       <c r="G267" s="152">
         <f>H230</f>
         <v>1450</v>
@@ -32089,10 +32089,10 @@
       <c r="H267" s="151" t="s">
         <v>465</v>
       </c>
-      <c r="I267" s="258" t="s">
+      <c r="I267" s="261" t="s">
         <v>466</v>
       </c>
-      <c r="J267" s="258"/>
+      <c r="J267" s="261"/>
       <c r="K267" s="170" t="s">
         <v>116</v>
       </c>
@@ -32108,28 +32108,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C58:J58"/>
-    <mergeCell ref="C22:J22"/>
-    <mergeCell ref="C159:J159"/>
-    <mergeCell ref="C177:J177"/>
-    <mergeCell ref="C197:J197"/>
-    <mergeCell ref="C212:J212"/>
-    <mergeCell ref="C227:J227"/>
-    <mergeCell ref="C238:J238"/>
-    <mergeCell ref="E261:F261"/>
-    <mergeCell ref="I261:J261"/>
+    <mergeCell ref="E265:F265"/>
+    <mergeCell ref="I265:J265"/>
+    <mergeCell ref="E266:F266"/>
+    <mergeCell ref="I266:J266"/>
+    <mergeCell ref="E267:F267"/>
+    <mergeCell ref="I267:J267"/>
     <mergeCell ref="E262:F262"/>
     <mergeCell ref="I262:J262"/>
     <mergeCell ref="E263:F263"/>
     <mergeCell ref="I263:J263"/>
     <mergeCell ref="E264:F264"/>
     <mergeCell ref="I264:J264"/>
-    <mergeCell ref="E265:F265"/>
-    <mergeCell ref="I265:J265"/>
-    <mergeCell ref="E266:F266"/>
-    <mergeCell ref="I266:J266"/>
-    <mergeCell ref="E267:F267"/>
-    <mergeCell ref="I267:J267"/>
+    <mergeCell ref="C212:J212"/>
+    <mergeCell ref="C227:J227"/>
+    <mergeCell ref="C238:J238"/>
+    <mergeCell ref="E261:F261"/>
+    <mergeCell ref="I261:J261"/>
+    <mergeCell ref="C58:J58"/>
+    <mergeCell ref="C22:J22"/>
+    <mergeCell ref="C159:J159"/>
+    <mergeCell ref="C177:J177"/>
+    <mergeCell ref="C197:J197"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -32204,43 +32204,43 @@
       <c r="AE1" s="236"/>
     </row>
     <row r="2" spans="2:31" ht="15" customHeight="1">
-      <c r="B2" s="262" t="s">
+      <c r="B2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="C2" s="262" t="s">
+      <c r="C2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="D2" s="262" t="s">
+      <c r="D2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="E2" s="262" t="s">
+      <c r="E2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="F2" s="262" t="s">
+      <c r="F2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="G2" s="262" t="s">
+      <c r="G2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="H2" s="262" t="s">
+      <c r="H2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="I2" s="262" t="s">
+      <c r="I2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="J2" s="262" t="s">
+      <c r="J2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="K2" s="262" t="s">
+      <c r="K2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="L2" s="262" t="s">
+      <c r="L2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="M2" s="262" t="s">
+      <c r="M2" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="N2" s="262" t="s">
+      <c r="N2" s="314" t="s">
         <v>472</v>
       </c>
       <c r="O2" s="227"/>
@@ -32280,43 +32280,43 @@
       <c r="AE2" s="236"/>
     </row>
     <row r="3" spans="2:31" ht="15" customHeight="1">
-      <c r="B3" s="262" t="s">
+      <c r="B3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="C3" s="262" t="s">
+      <c r="C3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="D3" s="262" t="s">
+      <c r="D3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="E3" s="262" t="s">
+      <c r="E3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="F3" s="262" t="s">
+      <c r="F3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="G3" s="262" t="s">
+      <c r="G3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="H3" s="262" t="s">
+      <c r="H3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="I3" s="262" t="s">
+      <c r="I3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="J3" s="262" t="s">
+      <c r="J3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="K3" s="262" t="s">
+      <c r="K3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="L3" s="262" t="s">
+      <c r="L3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="M3" s="262" t="s">
+      <c r="M3" s="314" t="s">
         <v>472</v>
       </c>
-      <c r="N3" s="262" t="s">
+      <c r="N3" s="314" t="s">
         <v>472</v>
       </c>
       <c r="O3" s="227"/>
@@ -32356,43 +32356,43 @@
       <c r="AE3" s="236"/>
     </row>
     <row r="4" spans="2:31" ht="15" customHeight="1">
-      <c r="B4" s="263" t="s">
+      <c r="B4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="C4" s="263" t="s">
+      <c r="C4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="D4" s="263" t="s">
+      <c r="D4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="E4" s="263" t="s">
+      <c r="E4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="F4" s="263" t="s">
+      <c r="F4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="G4" s="263" t="s">
+      <c r="G4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="H4" s="263" t="s">
+      <c r="H4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="I4" s="263" t="s">
+      <c r="I4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="J4" s="263" t="s">
+      <c r="J4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="K4" s="263" t="s">
+      <c r="K4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="L4" s="263" t="s">
+      <c r="L4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="M4" s="263" t="s">
+      <c r="M4" s="315" t="s">
         <v>476</v>
       </c>
-      <c r="N4" s="263" t="s">
+      <c r="N4" s="315" t="s">
         <v>476</v>
       </c>
       <c r="O4" s="227"/>
@@ -32482,43 +32482,43 @@
       <c r="AE5" s="236"/>
     </row>
     <row r="6" spans="2:31" ht="15" customHeight="1">
-      <c r="B6" s="264" t="s">
+      <c r="B6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="C6" s="264" t="s">
+      <c r="C6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="D6" s="264" t="s">
+      <c r="D6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="E6" s="264" t="s">
+      <c r="E6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="F6" s="264" t="s">
+      <c r="F6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="G6" s="264" t="s">
+      <c r="G6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="H6" s="264" t="s">
+      <c r="H6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="I6" s="264" t="s">
+      <c r="I6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="J6" s="264" t="s">
+      <c r="J6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="K6" s="264" t="s">
+      <c r="K6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="L6" s="264" t="s">
+      <c r="L6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="M6" s="264" t="s">
+      <c r="M6" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="N6" s="264" t="s">
+      <c r="N6" s="265" t="s">
         <v>481</v>
       </c>
       <c r="O6" s="227"/>
@@ -32937,43 +32937,43 @@
       <c r="AE14" s="227"/>
     </row>
     <row r="15" spans="2:31" ht="15" customHeight="1">
-      <c r="B15" s="264" t="s">
+      <c r="B15" s="265" t="s">
         <v>497</v>
       </c>
-      <c r="C15" s="264" t="s">
+      <c r="C15" s="265" t="s">
         <v>497</v>
       </c>
-      <c r="D15" s="264" t="s">
+      <c r="D15" s="265" t="s">
         <v>497</v>
       </c>
-      <c r="E15" s="264" t="s">
+      <c r="E15" s="265" t="s">
         <v>497</v>
       </c>
-      <c r="F15" s="264" t="s">
+      <c r="F15" s="265" t="s">
         <v>497</v>
       </c>
-      <c r="G15" s="264" t="s">
+      <c r="G15" s="265" t="s">
         <v>498</v>
       </c>
-      <c r="H15" s="264" t="s">
+      <c r="H15" s="265" t="s">
         <v>498</v>
       </c>
-      <c r="I15" s="264" t="s">
+      <c r="I15" s="265" t="s">
         <v>498</v>
       </c>
-      <c r="J15" s="264" t="s">
+      <c r="J15" s="265" t="s">
         <v>498</v>
       </c>
-      <c r="K15" s="264" t="s">
+      <c r="K15" s="265" t="s">
         <v>498</v>
       </c>
-      <c r="L15" s="264" t="s">
+      <c r="L15" s="265" t="s">
         <v>498</v>
       </c>
-      <c r="M15" s="264" t="s">
+      <c r="M15" s="265" t="s">
         <v>498</v>
       </c>
-      <c r="N15" s="264" t="s">
+      <c r="N15" s="265" t="s">
         <v>498</v>
       </c>
       <c r="O15" s="227"/>
@@ -32995,19 +32995,19 @@
       <c r="AE15" s="227"/>
     </row>
     <row r="16" spans="2:31" ht="15" customHeight="1">
-      <c r="B16" s="265" t="s">
+      <c r="B16" s="267" t="s">
         <v>499</v>
       </c>
-      <c r="C16" s="266" t="s">
+      <c r="C16" s="268" t="s">
         <v>499</v>
       </c>
-      <c r="D16" s="266" t="s">
+      <c r="D16" s="268" t="s">
         <v>499</v>
       </c>
-      <c r="E16" s="266" t="s">
+      <c r="E16" s="268" t="s">
         <v>499</v>
       </c>
-      <c r="F16" s="267" t="s">
+      <c r="F16" s="269" t="s">
         <v>499</v>
       </c>
       <c r="G16" s="227"/>
@@ -33037,19 +33037,19 @@
       <c r="AE16" s="227"/>
     </row>
     <row r="17" spans="2:31" ht="15" customHeight="1">
-      <c r="B17" s="268" t="s">
+      <c r="B17" s="270" t="s">
         <v>499</v>
       </c>
-      <c r="C17" s="269" t="s">
+      <c r="C17" s="271" t="s">
         <v>499</v>
       </c>
-      <c r="D17" s="269" t="s">
+      <c r="D17" s="271" t="s">
         <v>499</v>
       </c>
-      <c r="E17" s="269" t="s">
+      <c r="E17" s="271" t="s">
         <v>499</v>
       </c>
-      <c r="F17" s="270" t="s">
+      <c r="F17" s="272" t="s">
         <v>499</v>
       </c>
       <c r="G17" s="227"/>
@@ -33079,19 +33079,19 @@
       <c r="AE17" s="227"/>
     </row>
     <row r="18" spans="2:31" ht="15" customHeight="1">
-      <c r="B18" s="271" t="s">
+      <c r="B18" s="273" t="s">
         <v>499</v>
       </c>
-      <c r="C18" s="272" t="s">
+      <c r="C18" s="274" t="s">
         <v>499</v>
       </c>
-      <c r="D18" s="272" t="s">
+      <c r="D18" s="274" t="s">
         <v>499</v>
       </c>
-      <c r="E18" s="272" t="s">
+      <c r="E18" s="274" t="s">
         <v>499</v>
       </c>
-      <c r="F18" s="273" t="s">
+      <c r="F18" s="275" t="s">
         <v>499</v>
       </c>
       <c r="G18" s="227"/>
@@ -33121,19 +33121,19 @@
       <c r="AE18" s="227"/>
     </row>
     <row r="19" spans="2:31" ht="15" customHeight="1">
-      <c r="B19" s="274" t="s">
+      <c r="B19" s="276" t="s">
         <v>500</v>
       </c>
-      <c r="C19" s="275" t="s">
+      <c r="C19" s="277" t="s">
         <v>500</v>
       </c>
-      <c r="D19" s="275" t="s">
+      <c r="D19" s="277" t="s">
         <v>500</v>
       </c>
-      <c r="E19" s="275" t="s">
+      <c r="E19" s="277" t="s">
         <v>500</v>
       </c>
-      <c r="F19" s="276" t="s">
+      <c r="F19" s="278" t="s">
         <v>500</v>
       </c>
       <c r="G19" s="227"/>
@@ -33163,19 +33163,19 @@
       <c r="AE19" s="227"/>
     </row>
     <row r="20" spans="2:31" ht="15" customHeight="1">
-      <c r="B20" s="277" t="s">
+      <c r="B20" s="279" t="s">
         <v>500</v>
       </c>
-      <c r="C20" s="278" t="s">
+      <c r="C20" s="280" t="s">
         <v>500</v>
       </c>
-      <c r="D20" s="278" t="s">
+      <c r="D20" s="280" t="s">
         <v>500</v>
       </c>
-      <c r="E20" s="278" t="s">
+      <c r="E20" s="280" t="s">
         <v>500</v>
       </c>
-      <c r="F20" s="279" t="s">
+      <c r="F20" s="281" t="s">
         <v>500</v>
       </c>
       <c r="G20" s="227"/>
@@ -33205,19 +33205,19 @@
       <c r="AE20" s="227"/>
     </row>
     <row r="21" spans="2:31" ht="15" customHeight="1">
-      <c r="B21" s="280" t="s">
+      <c r="B21" s="282" t="s">
         <v>500</v>
       </c>
-      <c r="C21" s="281" t="s">
+      <c r="C21" s="283" t="s">
         <v>500</v>
       </c>
-      <c r="D21" s="281" t="s">
+      <c r="D21" s="283" t="s">
         <v>500</v>
       </c>
-      <c r="E21" s="281" t="s">
+      <c r="E21" s="283" t="s">
         <v>500</v>
       </c>
-      <c r="F21" s="282" t="s">
+      <c r="F21" s="284" t="s">
         <v>500</v>
       </c>
       <c r="G21" s="227"/>
@@ -33247,19 +33247,19 @@
       <c r="AE21" s="227"/>
     </row>
     <row r="22" spans="2:31" ht="15" customHeight="1">
-      <c r="B22" s="265" t="s">
+      <c r="B22" s="267" t="s">
         <v>501</v>
       </c>
-      <c r="C22" s="266" t="s">
+      <c r="C22" s="268" t="s">
         <v>501</v>
       </c>
-      <c r="D22" s="266" t="s">
+      <c r="D22" s="268" t="s">
         <v>501</v>
       </c>
-      <c r="E22" s="266" t="s">
+      <c r="E22" s="268" t="s">
         <v>501</v>
       </c>
-      <c r="F22" s="267" t="s">
+      <c r="F22" s="269" t="s">
         <v>501</v>
       </c>
       <c r="G22" s="227"/>
@@ -33289,19 +33289,19 @@
       <c r="AE22" s="227"/>
     </row>
     <row r="23" spans="2:31" ht="15" customHeight="1">
-      <c r="B23" s="268" t="s">
+      <c r="B23" s="270" t="s">
         <v>501</v>
       </c>
-      <c r="C23" s="269" t="s">
+      <c r="C23" s="271" t="s">
         <v>501</v>
       </c>
-      <c r="D23" s="269" t="s">
+      <c r="D23" s="271" t="s">
         <v>501</v>
       </c>
-      <c r="E23" s="269" t="s">
+      <c r="E23" s="271" t="s">
         <v>501</v>
       </c>
-      <c r="F23" s="270" t="s">
+      <c r="F23" s="272" t="s">
         <v>501</v>
       </c>
       <c r="G23" s="227"/>
@@ -33331,19 +33331,19 @@
       <c r="AE23" s="227"/>
     </row>
     <row r="24" spans="2:31" ht="15" customHeight="1">
-      <c r="B24" s="271" t="s">
+      <c r="B24" s="273" t="s">
         <v>501</v>
       </c>
-      <c r="C24" s="272" t="s">
+      <c r="C24" s="274" t="s">
         <v>501</v>
       </c>
-      <c r="D24" s="272" t="s">
+      <c r="D24" s="274" t="s">
         <v>501</v>
       </c>
-      <c r="E24" s="272" t="s">
+      <c r="E24" s="274" t="s">
         <v>501</v>
       </c>
-      <c r="F24" s="273" t="s">
+      <c r="F24" s="275" t="s">
         <v>501</v>
       </c>
       <c r="G24" s="227"/>
@@ -33373,19 +33373,19 @@
       <c r="AE24" s="227"/>
     </row>
     <row r="25" spans="2:31" ht="15" customHeight="1">
-      <c r="B25" s="283" t="s">
+      <c r="B25" s="285" t="s">
         <v>502</v>
       </c>
-      <c r="C25" s="284" t="s">
+      <c r="C25" s="286" t="s">
         <v>502</v>
       </c>
-      <c r="D25" s="284" t="s">
+      <c r="D25" s="286" t="s">
         <v>502</v>
       </c>
-      <c r="E25" s="284" t="s">
+      <c r="E25" s="286" t="s">
         <v>502</v>
       </c>
-      <c r="F25" s="285" t="s">
+      <c r="F25" s="287" t="s">
         <v>502</v>
       </c>
       <c r="G25" s="227"/>
@@ -33415,19 +33415,19 @@
       <c r="AE25" s="227"/>
     </row>
     <row r="26" spans="2:31" ht="15" customHeight="1">
-      <c r="B26" s="286" t="s">
+      <c r="B26" s="288" t="s">
         <v>502</v>
       </c>
-      <c r="C26" s="287" t="s">
+      <c r="C26" s="289" t="s">
         <v>502</v>
       </c>
-      <c r="D26" s="287" t="s">
+      <c r="D26" s="289" t="s">
         <v>502</v>
       </c>
-      <c r="E26" s="287" t="s">
+      <c r="E26" s="289" t="s">
         <v>502</v>
       </c>
-      <c r="F26" s="288" t="s">
+      <c r="F26" s="290" t="s">
         <v>502</v>
       </c>
       <c r="G26" s="227"/>
@@ -33457,19 +33457,19 @@
       <c r="AE26" s="227"/>
     </row>
     <row r="27" spans="2:31" ht="15" customHeight="1">
-      <c r="B27" s="289" t="s">
+      <c r="B27" s="291" t="s">
         <v>502</v>
       </c>
-      <c r="C27" s="290" t="s">
+      <c r="C27" s="292" t="s">
         <v>502</v>
       </c>
-      <c r="D27" s="290" t="s">
+      <c r="D27" s="292" t="s">
         <v>502</v>
       </c>
-      <c r="E27" s="290" t="s">
+      <c r="E27" s="292" t="s">
         <v>502</v>
       </c>
-      <c r="F27" s="291" t="s">
+      <c r="F27" s="293" t="s">
         <v>502</v>
       </c>
       <c r="G27" s="227"/>
@@ -33531,19 +33531,19 @@
       <c r="AE28" s="227"/>
     </row>
     <row r="29" spans="2:31" ht="15" customHeight="1">
-      <c r="B29" s="264" t="s">
+      <c r="B29" s="265" t="s">
         <v>503</v>
       </c>
-      <c r="C29" s="264" t="s">
+      <c r="C29" s="265" t="s">
         <v>503</v>
       </c>
-      <c r="D29" s="264" t="s">
+      <c r="D29" s="265" t="s">
         <v>503</v>
       </c>
-      <c r="E29" s="264" t="s">
+      <c r="E29" s="265" t="s">
         <v>503</v>
       </c>
-      <c r="F29" s="264" t="s">
+      <c r="F29" s="265" t="s">
         <v>503</v>
       </c>
       <c r="G29" s="227"/>
@@ -33768,28 +33768,28 @@
       <c r="F34" s="239" t="s">
         <v>509</v>
       </c>
-      <c r="G34" s="264" t="s">
+      <c r="G34" s="265" t="s">
         <v>510</v>
       </c>
-      <c r="H34" s="264" t="s">
+      <c r="H34" s="265" t="s">
         <v>510</v>
       </c>
-      <c r="I34" s="264" t="s">
+      <c r="I34" s="265" t="s">
         <v>510</v>
       </c>
-      <c r="J34" s="264" t="s">
+      <c r="J34" s="265" t="s">
         <v>510</v>
       </c>
-      <c r="K34" s="264" t="s">
+      <c r="K34" s="265" t="s">
         <v>510</v>
       </c>
-      <c r="L34" s="264" t="s">
+      <c r="L34" s="265" t="s">
         <v>510</v>
       </c>
-      <c r="M34" s="264" t="s">
+      <c r="M34" s="265" t="s">
         <v>510</v>
       </c>
-      <c r="N34" s="264" t="s">
+      <c r="N34" s="265" t="s">
         <v>510</v>
       </c>
       <c r="O34" s="227"/>
@@ -33829,17 +33829,17 @@
       <c r="F35" s="239" t="s">
         <v>512</v>
       </c>
-      <c r="G35" s="292" t="s">
+      <c r="G35" s="266" t="s">
         <v>387</v>
       </c>
-      <c r="H35" s="292"/>
-      <c r="I35" s="292"/>
-      <c r="J35" s="292"/>
-      <c r="K35" s="292"/>
-      <c r="L35" s="292" t="s">
+      <c r="H35" s="266"/>
+      <c r="I35" s="266"/>
+      <c r="J35" s="266"/>
+      <c r="K35" s="266"/>
+      <c r="L35" s="266" t="s">
         <v>513</v>
       </c>
-      <c r="M35" s="292"/>
+      <c r="M35" s="266"/>
       <c r="N35" s="244" t="s">
         <v>389</v>
       </c>
@@ -33880,18 +33880,18 @@
       <c r="F36" s="239" t="s">
         <v>515</v>
       </c>
-      <c r="G36" s="293" t="s">
+      <c r="G36" s="318" t="s">
         <v>516</v>
       </c>
-      <c r="H36" s="293"/>
-      <c r="I36" s="293"/>
-      <c r="J36" s="293"/>
-      <c r="K36" s="293"/>
-      <c r="L36" s="294">
+      <c r="H36" s="318"/>
+      <c r="I36" s="318"/>
+      <c r="J36" s="318"/>
+      <c r="K36" s="318"/>
+      <c r="L36" s="319">
         <f>Variance!D240</f>
         <v>534270.01039999991</v>
       </c>
-      <c r="M36" s="294"/>
+      <c r="M36" s="319"/>
       <c r="N36" s="246" t="s">
         <v>391</v>
       </c>
@@ -33919,18 +33919,18 @@
       <c r="D37" s="227"/>
       <c r="E37" s="227"/>
       <c r="F37" s="227"/>
-      <c r="G37" s="295" t="s">
+      <c r="G37" s="263" t="s">
         <v>517</v>
       </c>
-      <c r="H37" s="295"/>
-      <c r="I37" s="295"/>
-      <c r="J37" s="295"/>
-      <c r="K37" s="295"/>
-      <c r="L37" s="296">
+      <c r="H37" s="263"/>
+      <c r="I37" s="263"/>
+      <c r="J37" s="263"/>
+      <c r="K37" s="263"/>
+      <c r="L37" s="312">
         <f>Variance!D241</f>
         <v>-84994.689999999988</v>
       </c>
-      <c r="M37" s="296"/>
+      <c r="M37" s="312"/>
       <c r="N37" s="228" t="str">
         <f>Variance!E241</f>
         <v>Unfavorable</v>
@@ -33959,18 +33959,18 @@
       <c r="D38" s="227"/>
       <c r="E38" s="227"/>
       <c r="F38" s="227"/>
-      <c r="G38" s="295" t="s">
+      <c r="G38" s="263" t="s">
         <v>518</v>
       </c>
-      <c r="H38" s="295"/>
-      <c r="I38" s="295"/>
-      <c r="J38" s="295"/>
-      <c r="K38" s="295"/>
-      <c r="L38" s="296">
+      <c r="H38" s="263"/>
+      <c r="I38" s="263"/>
+      <c r="J38" s="263"/>
+      <c r="K38" s="263"/>
+      <c r="L38" s="312">
         <f>Variance!D242</f>
         <v>-17667.04999999989</v>
       </c>
-      <c r="M38" s="296"/>
+      <c r="M38" s="312"/>
       <c r="N38" s="228" t="str">
         <f>Variance!E242</f>
         <v>Unfavorable</v>
@@ -33999,18 +33999,18 @@
       <c r="D39" s="227"/>
       <c r="E39" s="227"/>
       <c r="F39" s="227"/>
-      <c r="G39" s="295" t="s">
+      <c r="G39" s="263" t="s">
         <v>519</v>
       </c>
-      <c r="H39" s="295"/>
-      <c r="I39" s="295"/>
-      <c r="J39" s="295"/>
-      <c r="K39" s="295"/>
-      <c r="L39" s="296">
+      <c r="H39" s="263"/>
+      <c r="I39" s="263"/>
+      <c r="J39" s="263"/>
+      <c r="K39" s="263"/>
+      <c r="L39" s="312">
         <f>Variance!D243</f>
         <v>4470</v>
       </c>
-      <c r="M39" s="296"/>
+      <c r="M39" s="312"/>
       <c r="N39" s="228" t="str">
         <f>Variance!E243</f>
         <v>Favorable</v>
@@ -34039,18 +34039,18 @@
       <c r="D40" s="227"/>
       <c r="E40" s="227"/>
       <c r="F40" s="227"/>
-      <c r="G40" s="295" t="s">
+      <c r="G40" s="263" t="s">
         <v>520</v>
       </c>
-      <c r="H40" s="295"/>
-      <c r="I40" s="295"/>
-      <c r="J40" s="295"/>
-      <c r="K40" s="295"/>
-      <c r="L40" s="296">
+      <c r="H40" s="263"/>
+      <c r="I40" s="263"/>
+      <c r="J40" s="263"/>
+      <c r="K40" s="263"/>
+      <c r="L40" s="312">
         <f>Variance!D244</f>
         <v>6289.58</v>
       </c>
-      <c r="M40" s="296"/>
+      <c r="M40" s="312"/>
       <c r="N40" s="228" t="str">
         <f>Variance!E244</f>
         <v>Favorable</v>
@@ -34079,18 +34079,18 @@
       <c r="D41" s="227"/>
       <c r="E41" s="227"/>
       <c r="F41" s="227"/>
-      <c r="G41" s="295" t="s">
+      <c r="G41" s="263" t="s">
         <v>521</v>
       </c>
-      <c r="H41" s="295"/>
-      <c r="I41" s="295"/>
-      <c r="J41" s="295"/>
-      <c r="K41" s="295"/>
-      <c r="L41" s="296">
+      <c r="H41" s="263"/>
+      <c r="I41" s="263"/>
+      <c r="J41" s="263"/>
+      <c r="K41" s="263"/>
+      <c r="L41" s="312">
         <f>Variance!D245</f>
         <v>-11327.579999999996</v>
       </c>
-      <c r="M41" s="296"/>
+      <c r="M41" s="312"/>
       <c r="N41" s="228" t="str">
         <f>Variance!E245</f>
         <v>Unfavorable</v>
@@ -34119,18 +34119,18 @@
       <c r="D42" s="227"/>
       <c r="E42" s="227"/>
       <c r="F42" s="227"/>
-      <c r="G42" s="295" t="s">
+      <c r="G42" s="263" t="s">
         <v>522</v>
       </c>
-      <c r="H42" s="295"/>
-      <c r="I42" s="295"/>
-      <c r="J42" s="295"/>
-      <c r="K42" s="295"/>
-      <c r="L42" s="296">
+      <c r="H42" s="263"/>
+      <c r="I42" s="263"/>
+      <c r="J42" s="263"/>
+      <c r="K42" s="263"/>
+      <c r="L42" s="312">
         <f>Variance!D246</f>
         <v>-4714.1199999999935</v>
       </c>
-      <c r="M42" s="296"/>
+      <c r="M42" s="312"/>
       <c r="N42" s="228" t="str">
         <f>Variance!E246</f>
         <v>Unfavorable</v>
@@ -34159,18 +34159,18 @@
       <c r="D43" s="227"/>
       <c r="E43" s="227"/>
       <c r="F43" s="227"/>
-      <c r="G43" s="295" t="s">
+      <c r="G43" s="263" t="s">
         <v>523</v>
       </c>
-      <c r="H43" s="295"/>
-      <c r="I43" s="295"/>
-      <c r="J43" s="295"/>
-      <c r="K43" s="295"/>
-      <c r="L43" s="296">
+      <c r="H43" s="263"/>
+      <c r="I43" s="263"/>
+      <c r="J43" s="263"/>
+      <c r="K43" s="263"/>
+      <c r="L43" s="312">
         <f>SUM(Variance!D247:D248)</f>
         <v>8649.6000000000131</v>
       </c>
-      <c r="M43" s="296"/>
+      <c r="M43" s="312"/>
       <c r="N43" s="228" t="str">
         <f>IF(L43&gt;0,"Favorable",IF(L43&lt;0,"Unfavorable","Neutral"))</f>
         <v>Favorable</v>
@@ -34199,18 +34199,18 @@
       <c r="D44" s="227"/>
       <c r="E44" s="227"/>
       <c r="F44" s="227"/>
-      <c r="G44" s="295" t="s">
+      <c r="G44" s="263" t="s">
         <v>524</v>
       </c>
-      <c r="H44" s="295"/>
-      <c r="I44" s="295"/>
-      <c r="J44" s="295"/>
-      <c r="K44" s="295"/>
-      <c r="L44" s="296">
+      <c r="H44" s="263"/>
+      <c r="I44" s="263"/>
+      <c r="J44" s="263"/>
+      <c r="K44" s="263"/>
+      <c r="L44" s="312">
         <f>Variance!D249</f>
         <v>3927.6695999999974</v>
       </c>
-      <c r="M44" s="296"/>
+      <c r="M44" s="312"/>
       <c r="N44" s="228" t="str">
         <f>Variance!E249</f>
         <v>Favorable</v>
@@ -34239,18 +34239,18 @@
       <c r="D45" s="227"/>
       <c r="E45" s="227"/>
       <c r="F45" s="227"/>
-      <c r="G45" s="295" t="s">
+      <c r="G45" s="263" t="s">
         <v>525</v>
       </c>
-      <c r="H45" s="295"/>
-      <c r="I45" s="295"/>
-      <c r="J45" s="295"/>
-      <c r="K45" s="295"/>
-      <c r="L45" s="296">
+      <c r="H45" s="263"/>
+      <c r="I45" s="263"/>
+      <c r="J45" s="263"/>
+      <c r="K45" s="263"/>
+      <c r="L45" s="312">
         <f>SUM(Variance!D250:D251)</f>
         <v>-800</v>
       </c>
-      <c r="M45" s="296"/>
+      <c r="M45" s="312"/>
       <c r="N45" s="228" t="str">
         <f>IF(L45&gt;0,"Favorable",IF(L45&lt;0,"Unfavorable","Neutral"))</f>
         <v>Unfavorable</v>
@@ -34279,18 +34279,18 @@
       <c r="D46" s="227"/>
       <c r="E46" s="227"/>
       <c r="F46" s="227"/>
-      <c r="G46" s="295" t="s">
+      <c r="G46" s="263" t="s">
         <v>526</v>
       </c>
-      <c r="H46" s="295"/>
-      <c r="I46" s="295"/>
-      <c r="J46" s="295"/>
-      <c r="K46" s="295"/>
-      <c r="L46" s="296">
+      <c r="H46" s="263"/>
+      <c r="I46" s="263"/>
+      <c r="J46" s="263"/>
+      <c r="K46" s="263"/>
+      <c r="L46" s="312">
         <f>SUM(Variance!D252:D253)</f>
         <v>-1760</v>
       </c>
-      <c r="M46" s="296"/>
+      <c r="M46" s="312"/>
       <c r="N46" s="228" t="str">
         <f>IF(L46&gt;0,"Favorable",IF(L46&lt;0,"Unfavorable","Neutral"))</f>
         <v>Unfavorable</v>
@@ -34319,18 +34319,18 @@
       <c r="D47" s="227"/>
       <c r="E47" s="227"/>
       <c r="F47" s="227"/>
-      <c r="G47" s="295" t="s">
+      <c r="G47" s="263" t="s">
         <v>527</v>
       </c>
-      <c r="H47" s="295"/>
-      <c r="I47" s="295"/>
-      <c r="J47" s="295"/>
-      <c r="K47" s="295"/>
-      <c r="L47" s="296">
+      <c r="H47" s="263"/>
+      <c r="I47" s="263"/>
+      <c r="J47" s="263"/>
+      <c r="K47" s="263"/>
+      <c r="L47" s="312">
         <f>Variance!D254</f>
         <v>17400</v>
       </c>
-      <c r="M47" s="296"/>
+      <c r="M47" s="312"/>
       <c r="N47" s="228" t="str">
         <f>Variance!E254</f>
         <v>Favorable</v>
@@ -34359,18 +34359,18 @@
       <c r="D48" s="227"/>
       <c r="E48" s="227"/>
       <c r="F48" s="227"/>
-      <c r="G48" s="297" t="s">
+      <c r="G48" s="316" t="s">
         <v>528</v>
       </c>
-      <c r="H48" s="297"/>
-      <c r="I48" s="297"/>
-      <c r="J48" s="297"/>
-      <c r="K48" s="297"/>
-      <c r="L48" s="298">
+      <c r="H48" s="316"/>
+      <c r="I48" s="316"/>
+      <c r="J48" s="316"/>
+      <c r="K48" s="316"/>
+      <c r="L48" s="317">
         <f>Variance!D256</f>
         <v>453743.42000000004</v>
       </c>
-      <c r="M48" s="298"/>
+      <c r="M48" s="317"/>
       <c r="N48" s="247" t="s">
         <v>407</v>
       </c>
@@ -34425,43 +34425,43 @@
       <c r="AE49" s="227"/>
     </row>
     <row r="50" spans="2:31" ht="15" customHeight="1">
-      <c r="B50" s="262" t="s">
+      <c r="B50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="C50" s="262" t="s">
+      <c r="C50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="D50" s="262" t="s">
+      <c r="D50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="E50" s="262" t="s">
+      <c r="E50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="F50" s="262" t="s">
+      <c r="F50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="G50" s="262" t="s">
+      <c r="G50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="H50" s="262" t="s">
+      <c r="H50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="I50" s="262" t="s">
+      <c r="I50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="J50" s="262" t="s">
+      <c r="J50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="K50" s="262" t="s">
+      <c r="K50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="L50" s="262" t="s">
+      <c r="L50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="M50" s="262" t="s">
+      <c r="M50" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="N50" s="262" t="s">
+      <c r="N50" s="314" t="s">
         <v>529</v>
       </c>
       <c r="O50" s="227"/>
@@ -34483,43 +34483,43 @@
       <c r="AE50" s="227"/>
     </row>
     <row r="51" spans="2:31" ht="15" customHeight="1">
-      <c r="B51" s="262" t="s">
+      <c r="B51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="C51" s="262" t="s">
+      <c r="C51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="D51" s="262" t="s">
+      <c r="D51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="E51" s="262" t="s">
+      <c r="E51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="F51" s="262" t="s">
+      <c r="F51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="G51" s="262" t="s">
+      <c r="G51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="H51" s="262" t="s">
+      <c r="H51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="I51" s="262" t="s">
+      <c r="I51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="J51" s="262" t="s">
+      <c r="J51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="K51" s="262" t="s">
+      <c r="K51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="L51" s="262" t="s">
+      <c r="L51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="M51" s="262" t="s">
+      <c r="M51" s="314" t="s">
         <v>529</v>
       </c>
-      <c r="N51" s="262" t="s">
+      <c r="N51" s="314" t="s">
         <v>529</v>
       </c>
       <c r="O51" s="227"/>
@@ -34541,43 +34541,43 @@
       <c r="AE51" s="227"/>
     </row>
     <row r="52" spans="2:31" ht="15" customHeight="1">
-      <c r="B52" s="263" t="s">
+      <c r="B52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="C52" s="263" t="s">
+      <c r="C52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="D52" s="263" t="s">
+      <c r="D52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="E52" s="263" t="s">
+      <c r="E52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="F52" s="263" t="s">
+      <c r="F52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="G52" s="263" t="s">
+      <c r="G52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="H52" s="263" t="s">
+      <c r="H52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="I52" s="263" t="s">
+      <c r="I52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="J52" s="263" t="s">
+      <c r="J52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="K52" s="263" t="s">
+      <c r="K52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="L52" s="263" t="s">
+      <c r="L52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="M52" s="263" t="s">
+      <c r="M52" s="315" t="s">
         <v>530</v>
       </c>
-      <c r="N52" s="263" t="s">
+      <c r="N52" s="315" t="s">
         <v>530</v>
       </c>
       <c r="O52" s="227"/>
@@ -34631,43 +34631,43 @@
       <c r="AE53" s="227"/>
     </row>
     <row r="54" spans="2:31" ht="15" customHeight="1">
-      <c r="B54" s="264" t="s">
+      <c r="B54" s="265" t="s">
         <v>531</v>
       </c>
-      <c r="C54" s="264" t="s">
+      <c r="C54" s="265" t="s">
         <v>531</v>
       </c>
-      <c r="D54" s="264" t="s">
+      <c r="D54" s="265" t="s">
         <v>531</v>
       </c>
-      <c r="E54" s="264" t="s">
+      <c r="E54" s="265" t="s">
         <v>531</v>
       </c>
-      <c r="F54" s="264" t="s">
+      <c r="F54" s="265" t="s">
         <v>531</v>
       </c>
-      <c r="G54" s="264" t="s">
+      <c r="G54" s="265" t="s">
         <v>531</v>
       </c>
-      <c r="H54" s="264" t="s">
+      <c r="H54" s="265" t="s">
         <v>532</v>
       </c>
-      <c r="I54" s="264" t="s">
+      <c r="I54" s="265" t="s">
         <v>532</v>
       </c>
-      <c r="J54" s="264" t="s">
+      <c r="J54" s="265" t="s">
         <v>532</v>
       </c>
-      <c r="K54" s="264" t="s">
+      <c r="K54" s="265" t="s">
         <v>532</v>
       </c>
-      <c r="L54" s="264" t="s">
+      <c r="L54" s="265" t="s">
         <v>532</v>
       </c>
-      <c r="M54" s="264" t="s">
+      <c r="M54" s="265" t="s">
         <v>532</v>
       </c>
-      <c r="N54" s="264" t="s">
+      <c r="N54" s="265" t="s">
         <v>532</v>
       </c>
       <c r="O54" s="227"/>
@@ -34688,7 +34688,7 @@
       <c r="AD54" s="227"/>
       <c r="AE54" s="227"/>
     </row>
-    <row r="55" spans="2:31" ht="15" customHeight="1">
+    <row r="55" spans="2:31" ht="23.25">
       <c r="B55" s="244" t="s">
         <v>218</v>
       </c>
@@ -34711,14 +34711,14 @@
       <c r="I55" s="244" t="s">
         <v>225</v>
       </c>
-      <c r="J55" s="292" t="s">
+      <c r="J55" s="266" t="s">
         <v>228</v>
       </c>
-      <c r="K55" s="292"/>
-      <c r="L55" s="292" t="s">
+      <c r="K55" s="266"/>
+      <c r="L55" s="266" t="s">
         <v>535</v>
       </c>
-      <c r="M55" s="292"/>
+      <c r="M55" s="266"/>
       <c r="N55" s="244" t="s">
         <v>536</v>
       </c>
@@ -34767,16 +34767,16 @@
         <f>Forecast!D10</f>
         <v>0.69243835616438354</v>
       </c>
-      <c r="J56" s="296">
+      <c r="J56" s="312">
         <f>Forecast!D12</f>
         <v>4044921.5799999996</v>
       </c>
-      <c r="K56" s="296"/>
-      <c r="L56" s="296">
+      <c r="K56" s="312"/>
+      <c r="L56" s="312">
         <f>Forecast!D16</f>
         <v>1279795.4142999998</v>
       </c>
-      <c r="M56" s="296"/>
+      <c r="M56" s="312"/>
       <c r="N56" s="230">
         <f>Forecast!D17</f>
         <v>0.31639560594398469</v>
@@ -34826,16 +34826,16 @@
         <f>Forecast!E10</f>
         <v>0.67172602739726028</v>
       </c>
-      <c r="J57" s="299">
+      <c r="J57" s="313">
         <f>Forecast!E12</f>
         <v>3903659.3724999996</v>
       </c>
-      <c r="K57" s="299"/>
-      <c r="L57" s="299">
+      <c r="K57" s="313"/>
+      <c r="L57" s="313">
         <f>Forecast!E16</f>
         <v>1137547.1776000001</v>
       </c>
-      <c r="M57" s="299"/>
+      <c r="M57" s="313"/>
       <c r="N57" s="248">
         <f>Forecast!E17</f>
         <v>0.29140533767204357</v>
@@ -34885,16 +34885,16 @@
         <f>Forecast!G10</f>
         <v>0.68082191780821921</v>
       </c>
-      <c r="J58" s="296">
+      <c r="J58" s="312">
         <f>Forecast!G12</f>
         <v>3974207.8951500002</v>
       </c>
-      <c r="K58" s="296"/>
-      <c r="L58" s="296">
+      <c r="K58" s="312"/>
+      <c r="L58" s="312">
         <f>Forecast!G16</f>
         <v>1198073.9668440002</v>
       </c>
-      <c r="M58" s="296"/>
+      <c r="M58" s="312"/>
       <c r="N58" s="230">
         <f>Forecast!G17</f>
         <v>0.30146232870859435</v>
@@ -34944,16 +34944,16 @@
         <f>Forecast!I10</f>
         <v>0.65531506849315069</v>
       </c>
-      <c r="J59" s="296">
+      <c r="J59" s="312">
         <f>Forecast!I12</f>
         <v>3777975.0359500004</v>
       </c>
-      <c r="K59" s="296"/>
-      <c r="L59" s="296">
+      <c r="K59" s="312"/>
+      <c r="L59" s="312">
         <f>Forecast!I16</f>
         <v>1031710.4770119999</v>
       </c>
-      <c r="M59" s="296"/>
+      <c r="M59" s="312"/>
       <c r="N59" s="230">
         <f>Forecast!I17</f>
         <v>0.27308557287821478</v>
@@ -35009,43 +35009,43 @@
       <c r="AE60" s="227"/>
     </row>
     <row r="61" spans="2:31" ht="15" customHeight="1">
-      <c r="B61" s="264" t="s">
+      <c r="B61" s="265" t="s">
         <v>541</v>
       </c>
-      <c r="C61" s="264" t="s">
+      <c r="C61" s="265" t="s">
         <v>541</v>
       </c>
-      <c r="D61" s="264" t="s">
+      <c r="D61" s="265" t="s">
         <v>541</v>
       </c>
-      <c r="E61" s="264" t="s">
+      <c r="E61" s="265" t="s">
         <v>541</v>
       </c>
-      <c r="F61" s="264" t="s">
+      <c r="F61" s="265" t="s">
         <v>541</v>
       </c>
-      <c r="G61" s="264" t="s">
+      <c r="G61" s="265" t="s">
         <v>541</v>
       </c>
-      <c r="H61" s="264" t="s">
+      <c r="H61" s="265" t="s">
         <v>542</v>
       </c>
-      <c r="I61" s="264" t="s">
+      <c r="I61" s="265" t="s">
         <v>542</v>
       </c>
-      <c r="J61" s="264" t="s">
+      <c r="J61" s="265" t="s">
         <v>542</v>
       </c>
-      <c r="K61" s="264" t="s">
+      <c r="K61" s="265" t="s">
         <v>542</v>
       </c>
-      <c r="L61" s="264" t="s">
+      <c r="L61" s="265" t="s">
         <v>542</v>
       </c>
-      <c r="M61" s="264" t="s">
+      <c r="M61" s="265" t="s">
         <v>542</v>
       </c>
-      <c r="N61" s="264" t="s">
+      <c r="N61" s="265" t="s">
         <v>542</v>
       </c>
       <c r="O61" s="227"/>
@@ -35579,43 +35579,43 @@
       <c r="AE77" s="227"/>
     </row>
     <row r="78" spans="2:31" ht="15" customHeight="1">
-      <c r="B78" s="264" t="s">
+      <c r="B78" s="265" t="s">
         <v>543</v>
       </c>
-      <c r="C78" s="264" t="s">
+      <c r="C78" s="265" t="s">
         <v>543</v>
       </c>
-      <c r="D78" s="264" t="s">
+      <c r="D78" s="265" t="s">
         <v>543</v>
       </c>
-      <c r="E78" s="264" t="s">
+      <c r="E78" s="265" t="s">
         <v>543</v>
       </c>
-      <c r="F78" s="264" t="s">
+      <c r="F78" s="265" t="s">
         <v>543</v>
       </c>
-      <c r="G78" s="264" t="s">
+      <c r="G78" s="265" t="s">
         <v>543</v>
       </c>
-      <c r="H78" s="264" t="s">
+      <c r="H78" s="265" t="s">
         <v>543</v>
       </c>
-      <c r="I78" s="264" t="s">
+      <c r="I78" s="265" t="s">
         <v>544</v>
       </c>
-      <c r="J78" s="264" t="s">
+      <c r="J78" s="265" t="s">
         <v>544</v>
       </c>
-      <c r="K78" s="264" t="s">
+      <c r="K78" s="265" t="s">
         <v>544</v>
       </c>
-      <c r="L78" s="264" t="s">
+      <c r="L78" s="265" t="s">
         <v>544</v>
       </c>
-      <c r="M78" s="264" t="s">
+      <c r="M78" s="265" t="s">
         <v>544</v>
       </c>
-      <c r="N78" s="264" t="s">
+      <c r="N78" s="265" t="s">
         <v>544</v>
       </c>
       <c r="O78" s="227"/>
@@ -35637,43 +35637,43 @@
       <c r="AE78" s="227"/>
     </row>
     <row r="79" spans="2:31" ht="15" customHeight="1">
-      <c r="B79" s="265" t="s">
+      <c r="B79" s="267" t="s">
         <v>545</v>
       </c>
-      <c r="C79" s="266" t="s">
+      <c r="C79" s="268" t="s">
         <v>545</v>
       </c>
-      <c r="D79" s="266" t="s">
+      <c r="D79" s="268" t="s">
         <v>545</v>
       </c>
-      <c r="E79" s="266" t="s">
+      <c r="E79" s="268" t="s">
         <v>545</v>
       </c>
-      <c r="F79" s="266" t="s">
+      <c r="F79" s="268" t="s">
         <v>545</v>
       </c>
-      <c r="G79" s="266" t="s">
+      <c r="G79" s="268" t="s">
         <v>545</v>
       </c>
-      <c r="H79" s="267" t="s">
+      <c r="H79" s="269" t="s">
         <v>545</v>
       </c>
-      <c r="I79" s="300" t="s">
+      <c r="I79" s="294" t="s">
         <v>546</v>
       </c>
-      <c r="J79" s="301" t="s">
+      <c r="J79" s="295" t="s">
         <v>546</v>
       </c>
-      <c r="K79" s="301" t="s">
+      <c r="K79" s="295" t="s">
         <v>546</v>
       </c>
-      <c r="L79" s="301" t="s">
+      <c r="L79" s="295" t="s">
         <v>546</v>
       </c>
-      <c r="M79" s="301" t="s">
+      <c r="M79" s="295" t="s">
         <v>546</v>
       </c>
-      <c r="N79" s="302" t="s">
+      <c r="N79" s="296" t="s">
         <v>546</v>
       </c>
       <c r="O79" s="227"/>
@@ -35695,43 +35695,43 @@
       <c r="AE79" s="227"/>
     </row>
     <row r="80" spans="2:31" ht="15" customHeight="1">
-      <c r="B80" s="268" t="s">
+      <c r="B80" s="270" t="s">
         <v>545</v>
       </c>
-      <c r="C80" s="269" t="s">
+      <c r="C80" s="271" t="s">
         <v>545</v>
       </c>
-      <c r="D80" s="269" t="s">
+      <c r="D80" s="271" t="s">
         <v>545</v>
       </c>
-      <c r="E80" s="269" t="s">
+      <c r="E80" s="271" t="s">
         <v>545</v>
       </c>
-      <c r="F80" s="269" t="s">
+      <c r="F80" s="271" t="s">
         <v>545</v>
       </c>
-      <c r="G80" s="269" t="s">
+      <c r="G80" s="271" t="s">
         <v>545</v>
       </c>
-      <c r="H80" s="270" t="s">
+      <c r="H80" s="272" t="s">
         <v>545</v>
       </c>
-      <c r="I80" s="303" t="s">
+      <c r="I80" s="297" t="s">
         <v>546</v>
       </c>
-      <c r="J80" s="304" t="s">
+      <c r="J80" s="298" t="s">
         <v>546</v>
       </c>
-      <c r="K80" s="304" t="s">
+      <c r="K80" s="298" t="s">
         <v>546</v>
       </c>
-      <c r="L80" s="304" t="s">
+      <c r="L80" s="298" t="s">
         <v>546</v>
       </c>
-      <c r="M80" s="304" t="s">
+      <c r="M80" s="298" t="s">
         <v>546</v>
       </c>
-      <c r="N80" s="305" t="s">
+      <c r="N80" s="299" t="s">
         <v>546</v>
       </c>
       <c r="O80" s="227"/>
@@ -35753,43 +35753,43 @@
       <c r="AE80" s="227"/>
     </row>
     <row r="81" spans="2:31" ht="15" customHeight="1">
-      <c r="B81" s="271" t="s">
+      <c r="B81" s="273" t="s">
         <v>545</v>
       </c>
-      <c r="C81" s="272" t="s">
+      <c r="C81" s="274" t="s">
         <v>545</v>
       </c>
-      <c r="D81" s="272" t="s">
+      <c r="D81" s="274" t="s">
         <v>545</v>
       </c>
-      <c r="E81" s="272" t="s">
+      <c r="E81" s="274" t="s">
         <v>545</v>
       </c>
-      <c r="F81" s="272" t="s">
+      <c r="F81" s="274" t="s">
         <v>545</v>
       </c>
-      <c r="G81" s="272" t="s">
+      <c r="G81" s="274" t="s">
         <v>545</v>
       </c>
-      <c r="H81" s="273" t="s">
+      <c r="H81" s="275" t="s">
         <v>545</v>
       </c>
-      <c r="I81" s="306" t="s">
+      <c r="I81" s="300" t="s">
         <v>546</v>
       </c>
-      <c r="J81" s="307" t="s">
+      <c r="J81" s="301" t="s">
         <v>546</v>
       </c>
-      <c r="K81" s="307" t="s">
+      <c r="K81" s="301" t="s">
         <v>546</v>
       </c>
-      <c r="L81" s="307" t="s">
+      <c r="L81" s="301" t="s">
         <v>546</v>
       </c>
-      <c r="M81" s="307" t="s">
+      <c r="M81" s="301" t="s">
         <v>546</v>
       </c>
-      <c r="N81" s="308" t="s">
+      <c r="N81" s="302" t="s">
         <v>546</v>
       </c>
       <c r="O81" s="227"/>
@@ -35811,43 +35811,43 @@
       <c r="AE81" s="227"/>
     </row>
     <row r="82" spans="2:31" ht="15" customHeight="1">
-      <c r="B82" s="274" t="s">
+      <c r="B82" s="276" t="s">
         <v>547</v>
       </c>
-      <c r="C82" s="275" t="s">
+      <c r="C82" s="277" t="s">
         <v>547</v>
       </c>
-      <c r="D82" s="275" t="s">
+      <c r="D82" s="277" t="s">
         <v>547</v>
       </c>
-      <c r="E82" s="275" t="s">
+      <c r="E82" s="277" t="s">
         <v>547</v>
       </c>
-      <c r="F82" s="275" t="s">
+      <c r="F82" s="277" t="s">
         <v>547</v>
       </c>
-      <c r="G82" s="275" t="s">
+      <c r="G82" s="277" t="s">
         <v>547</v>
       </c>
-      <c r="H82" s="276" t="s">
+      <c r="H82" s="278" t="s">
         <v>547</v>
       </c>
-      <c r="I82" s="300" t="s">
+      <c r="I82" s="294" t="s">
         <v>548</v>
       </c>
-      <c r="J82" s="301" t="s">
+      <c r="J82" s="295" t="s">
         <v>548</v>
       </c>
-      <c r="K82" s="301" t="s">
+      <c r="K82" s="295" t="s">
         <v>548</v>
       </c>
-      <c r="L82" s="301" t="s">
+      <c r="L82" s="295" t="s">
         <v>548</v>
       </c>
-      <c r="M82" s="301" t="s">
+      <c r="M82" s="295" t="s">
         <v>548</v>
       </c>
-      <c r="N82" s="302" t="s">
+      <c r="N82" s="296" t="s">
         <v>548</v>
       </c>
       <c r="O82" s="227"/>
@@ -35869,43 +35869,43 @@
       <c r="AE82" s="227"/>
     </row>
     <row r="83" spans="2:31" ht="15" customHeight="1">
-      <c r="B83" s="277" t="s">
+      <c r="B83" s="279" t="s">
         <v>547</v>
       </c>
-      <c r="C83" s="278" t="s">
+      <c r="C83" s="280" t="s">
         <v>547</v>
       </c>
-      <c r="D83" s="278" t="s">
+      <c r="D83" s="280" t="s">
         <v>547</v>
       </c>
-      <c r="E83" s="278" t="s">
+      <c r="E83" s="280" t="s">
         <v>547</v>
       </c>
-      <c r="F83" s="278" t="s">
+      <c r="F83" s="280" t="s">
         <v>547</v>
       </c>
-      <c r="G83" s="278" t="s">
+      <c r="G83" s="280" t="s">
         <v>547</v>
       </c>
-      <c r="H83" s="279" t="s">
+      <c r="H83" s="281" t="s">
         <v>547</v>
       </c>
-      <c r="I83" s="303" t="s">
+      <c r="I83" s="297" t="s">
         <v>548</v>
       </c>
-      <c r="J83" s="304" t="s">
+      <c r="J83" s="298" t="s">
         <v>548</v>
       </c>
-      <c r="K83" s="304" t="s">
+      <c r="K83" s="298" t="s">
         <v>548</v>
       </c>
-      <c r="L83" s="304" t="s">
+      <c r="L83" s="298" t="s">
         <v>548</v>
       </c>
-      <c r="M83" s="304" t="s">
+      <c r="M83" s="298" t="s">
         <v>548</v>
       </c>
-      <c r="N83" s="305" t="s">
+      <c r="N83" s="299" t="s">
         <v>548</v>
       </c>
       <c r="O83" s="227"/>
@@ -35927,43 +35927,43 @@
       <c r="AE83" s="227"/>
     </row>
     <row r="84" spans="2:31" ht="15" customHeight="1">
-      <c r="B84" s="280" t="s">
+      <c r="B84" s="282" t="s">
         <v>547</v>
       </c>
-      <c r="C84" s="281" t="s">
+      <c r="C84" s="283" t="s">
         <v>547</v>
       </c>
-      <c r="D84" s="281" t="s">
+      <c r="D84" s="283" t="s">
         <v>547</v>
       </c>
-      <c r="E84" s="281" t="s">
+      <c r="E84" s="283" t="s">
         <v>547</v>
       </c>
-      <c r="F84" s="281" t="s">
+      <c r="F84" s="283" t="s">
         <v>547</v>
       </c>
-      <c r="G84" s="281" t="s">
+      <c r="G84" s="283" t="s">
         <v>547</v>
       </c>
-      <c r="H84" s="282" t="s">
+      <c r="H84" s="284" t="s">
         <v>547</v>
       </c>
-      <c r="I84" s="306" t="s">
+      <c r="I84" s="300" t="s">
         <v>548</v>
       </c>
-      <c r="J84" s="307" t="s">
+      <c r="J84" s="301" t="s">
         <v>548</v>
       </c>
-      <c r="K84" s="307" t="s">
+      <c r="K84" s="301" t="s">
         <v>548</v>
       </c>
-      <c r="L84" s="307" t="s">
+      <c r="L84" s="301" t="s">
         <v>548</v>
       </c>
-      <c r="M84" s="307" t="s">
+      <c r="M84" s="301" t="s">
         <v>548</v>
       </c>
-      <c r="N84" s="308" t="s">
+      <c r="N84" s="302" t="s">
         <v>548</v>
       </c>
       <c r="O84" s="227"/>
@@ -35985,43 +35985,43 @@
       <c r="AE84" s="227"/>
     </row>
     <row r="85" spans="2:31" ht="15" customHeight="1">
-      <c r="B85" s="283" t="s">
+      <c r="B85" s="285" t="s">
         <v>549</v>
       </c>
-      <c r="C85" s="284" t="s">
+      <c r="C85" s="286" t="s">
         <v>549</v>
       </c>
-      <c r="D85" s="284" t="s">
+      <c r="D85" s="286" t="s">
         <v>549</v>
       </c>
-      <c r="E85" s="284" t="s">
+      <c r="E85" s="286" t="s">
         <v>549</v>
       </c>
-      <c r="F85" s="284" t="s">
+      <c r="F85" s="286" t="s">
         <v>549</v>
       </c>
-      <c r="G85" s="284" t="s">
+      <c r="G85" s="286" t="s">
         <v>549</v>
       </c>
-      <c r="H85" s="285" t="s">
+      <c r="H85" s="287" t="s">
         <v>549</v>
       </c>
-      <c r="I85" s="309" t="s">
+      <c r="I85" s="303" t="s">
         <v>550</v>
       </c>
-      <c r="J85" s="310" t="s">
+      <c r="J85" s="304" t="s">
         <v>550</v>
       </c>
-      <c r="K85" s="310" t="s">
+      <c r="K85" s="304" t="s">
         <v>550</v>
       </c>
-      <c r="L85" s="310" t="s">
+      <c r="L85" s="304" t="s">
         <v>550</v>
       </c>
-      <c r="M85" s="310" t="s">
+      <c r="M85" s="304" t="s">
         <v>550</v>
       </c>
-      <c r="N85" s="311" t="s">
+      <c r="N85" s="305" t="s">
         <v>550</v>
       </c>
       <c r="O85" s="227"/>
@@ -36043,43 +36043,43 @@
       <c r="AE85" s="227"/>
     </row>
     <row r="86" spans="2:31" ht="15" customHeight="1">
-      <c r="B86" s="286" t="s">
+      <c r="B86" s="288" t="s">
         <v>549</v>
       </c>
-      <c r="C86" s="287" t="s">
+      <c r="C86" s="289" t="s">
         <v>549</v>
       </c>
-      <c r="D86" s="287" t="s">
+      <c r="D86" s="289" t="s">
         <v>549</v>
       </c>
-      <c r="E86" s="287" t="s">
+      <c r="E86" s="289" t="s">
         <v>549</v>
       </c>
-      <c r="F86" s="287" t="s">
+      <c r="F86" s="289" t="s">
         <v>549</v>
       </c>
-      <c r="G86" s="287" t="s">
+      <c r="G86" s="289" t="s">
         <v>549</v>
       </c>
-      <c r="H86" s="288" t="s">
+      <c r="H86" s="290" t="s">
         <v>549</v>
       </c>
-      <c r="I86" s="312" t="s">
+      <c r="I86" s="306" t="s">
         <v>550</v>
       </c>
-      <c r="J86" s="313" t="s">
+      <c r="J86" s="307" t="s">
         <v>550</v>
       </c>
-      <c r="K86" s="313" t="s">
+      <c r="K86" s="307" t="s">
         <v>550</v>
       </c>
-      <c r="L86" s="313" t="s">
+      <c r="L86" s="307" t="s">
         <v>550</v>
       </c>
-      <c r="M86" s="313" t="s">
+      <c r="M86" s="307" t="s">
         <v>550</v>
       </c>
-      <c r="N86" s="314" t="s">
+      <c r="N86" s="308" t="s">
         <v>550</v>
       </c>
       <c r="O86" s="227"/>
@@ -36101,43 +36101,43 @@
       <c r="AE86" s="227"/>
     </row>
     <row r="87" spans="2:31" ht="15" customHeight="1">
-      <c r="B87" s="289" t="s">
+      <c r="B87" s="291" t="s">
         <v>549</v>
       </c>
-      <c r="C87" s="290" t="s">
+      <c r="C87" s="292" t="s">
         <v>549</v>
       </c>
-      <c r="D87" s="290" t="s">
+      <c r="D87" s="292" t="s">
         <v>549</v>
       </c>
-      <c r="E87" s="290" t="s">
+      <c r="E87" s="292" t="s">
         <v>549</v>
       </c>
-      <c r="F87" s="290" t="s">
+      <c r="F87" s="292" t="s">
         <v>549</v>
       </c>
-      <c r="G87" s="290" t="s">
+      <c r="G87" s="292" t="s">
         <v>549</v>
       </c>
-      <c r="H87" s="291" t="s">
+      <c r="H87" s="293" t="s">
         <v>549</v>
       </c>
-      <c r="I87" s="315" t="s">
+      <c r="I87" s="309" t="s">
         <v>550</v>
       </c>
-      <c r="J87" s="316" t="s">
+      <c r="J87" s="310" t="s">
         <v>550</v>
       </c>
-      <c r="K87" s="316" t="s">
+      <c r="K87" s="310" t="s">
         <v>550</v>
       </c>
-      <c r="L87" s="316" t="s">
+      <c r="L87" s="310" t="s">
         <v>550</v>
       </c>
-      <c r="M87" s="316" t="s">
+      <c r="M87" s="310" t="s">
         <v>550</v>
       </c>
-      <c r="N87" s="317" t="s">
+      <c r="N87" s="311" t="s">
         <v>550</v>
       </c>
       <c r="O87" s="227"/>
@@ -36191,43 +36191,43 @@
       <c r="AE88" s="227"/>
     </row>
     <row r="89" spans="2:31" ht="15" customHeight="1">
-      <c r="B89" s="264" t="s">
+      <c r="B89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="C89" s="264" t="s">
+      <c r="C89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="D89" s="264" t="s">
+      <c r="D89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="E89" s="264" t="s">
+      <c r="E89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="F89" s="264" t="s">
+      <c r="F89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="G89" s="264" t="s">
+      <c r="G89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="H89" s="264" t="s">
+      <c r="H89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="I89" s="264" t="s">
+      <c r="I89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="J89" s="264" t="s">
+      <c r="J89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="K89" s="264" t="s">
+      <c r="K89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="L89" s="264" t="s">
+      <c r="L89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="M89" s="264" t="s">
+      <c r="M89" s="265" t="s">
         <v>551</v>
       </c>
-      <c r="N89" s="264" t="s">
+      <c r="N89" s="265" t="s">
         <v>551</v>
       </c>
       <c r="O89" s="227"/>
@@ -36252,23 +36252,23 @@
       <c r="B90" s="244" t="s">
         <v>552</v>
       </c>
-      <c r="C90" s="292" t="s">
+      <c r="C90" s="266" t="s">
         <v>553</v>
       </c>
-      <c r="D90" s="292"/>
-      <c r="E90" s="292"/>
-      <c r="F90" s="292"/>
-      <c r="G90" s="292"/>
-      <c r="H90" s="292"/>
-      <c r="I90" s="292"/>
-      <c r="J90" s="292" t="s">
+      <c r="D90" s="266"/>
+      <c r="E90" s="266"/>
+      <c r="F90" s="266"/>
+      <c r="G90" s="266"/>
+      <c r="H90" s="266"/>
+      <c r="I90" s="266"/>
+      <c r="J90" s="266" t="s">
         <v>554</v>
       </c>
-      <c r="K90" s="292"/>
-      <c r="L90" s="292" t="s">
+      <c r="K90" s="266"/>
+      <c r="L90" s="266" t="s">
         <v>459</v>
       </c>
-      <c r="M90" s="292"/>
+      <c r="M90" s="266"/>
       <c r="N90" s="244" t="s">
         <v>555</v>
       </c>
@@ -36294,23 +36294,23 @@
       <c r="B91" s="228">
         <v>1</v>
       </c>
-      <c r="C91" s="318" t="s">
+      <c r="C91" s="262" t="s">
         <v>556</v>
       </c>
-      <c r="D91" s="318"/>
-      <c r="E91" s="318"/>
-      <c r="F91" s="318"/>
-      <c r="G91" s="318"/>
-      <c r="H91" s="318"/>
-      <c r="I91" s="318"/>
-      <c r="J91" s="295" t="s">
+      <c r="D91" s="262"/>
+      <c r="E91" s="262"/>
+      <c r="F91" s="262"/>
+      <c r="G91" s="262"/>
+      <c r="H91" s="262"/>
+      <c r="I91" s="262"/>
+      <c r="J91" s="263" t="s">
         <v>557</v>
       </c>
-      <c r="K91" s="295"/>
-      <c r="L91" s="295" t="s">
+      <c r="K91" s="263"/>
+      <c r="L91" s="263" t="s">
         <v>558</v>
       </c>
-      <c r="M91" s="295"/>
+      <c r="M91" s="263"/>
       <c r="N91" s="239" t="s">
         <v>559</v>
       </c>
@@ -36336,23 +36336,23 @@
       <c r="B92" s="228">
         <v>2</v>
       </c>
-      <c r="C92" s="318" t="s">
+      <c r="C92" s="262" t="s">
         <v>560</v>
       </c>
-      <c r="D92" s="318"/>
-      <c r="E92" s="318"/>
-      <c r="F92" s="318"/>
-      <c r="G92" s="318"/>
-      <c r="H92" s="318"/>
-      <c r="I92" s="318"/>
-      <c r="J92" s="295" t="s">
+      <c r="D92" s="262"/>
+      <c r="E92" s="262"/>
+      <c r="F92" s="262"/>
+      <c r="G92" s="262"/>
+      <c r="H92" s="262"/>
+      <c r="I92" s="262"/>
+      <c r="J92" s="263" t="s">
         <v>561</v>
       </c>
-      <c r="K92" s="295"/>
-      <c r="L92" s="295" t="s">
+      <c r="K92" s="263"/>
+      <c r="L92" s="263" t="s">
         <v>562</v>
       </c>
-      <c r="M92" s="295"/>
+      <c r="M92" s="263"/>
       <c r="N92" s="239" t="s">
         <v>563</v>
       </c>
@@ -36378,23 +36378,23 @@
       <c r="B93" s="228">
         <v>3</v>
       </c>
-      <c r="C93" s="318" t="s">
+      <c r="C93" s="262" t="s">
         <v>564</v>
       </c>
-      <c r="D93" s="318"/>
-      <c r="E93" s="318"/>
-      <c r="F93" s="318"/>
-      <c r="G93" s="318"/>
-      <c r="H93" s="318"/>
-      <c r="I93" s="318"/>
-      <c r="J93" s="295" t="s">
+      <c r="D93" s="262"/>
+      <c r="E93" s="262"/>
+      <c r="F93" s="262"/>
+      <c r="G93" s="262"/>
+      <c r="H93" s="262"/>
+      <c r="I93" s="262"/>
+      <c r="J93" s="263" t="s">
         <v>565</v>
       </c>
-      <c r="K93" s="295"/>
-      <c r="L93" s="295" t="s">
+      <c r="K93" s="263"/>
+      <c r="L93" s="263" t="s">
         <v>566</v>
       </c>
-      <c r="M93" s="295"/>
+      <c r="M93" s="263"/>
       <c r="N93" s="239" t="s">
         <v>567</v>
       </c>
@@ -36420,23 +36420,23 @@
       <c r="B94" s="228">
         <v>4</v>
       </c>
-      <c r="C94" s="318" t="s">
+      <c r="C94" s="262" t="s">
         <v>568</v>
       </c>
-      <c r="D94" s="318"/>
-      <c r="E94" s="318"/>
-      <c r="F94" s="318"/>
-      <c r="G94" s="318"/>
-      <c r="H94" s="318"/>
-      <c r="I94" s="318"/>
-      <c r="J94" s="295" t="s">
+      <c r="D94" s="262"/>
+      <c r="E94" s="262"/>
+      <c r="F94" s="262"/>
+      <c r="G94" s="262"/>
+      <c r="H94" s="262"/>
+      <c r="I94" s="262"/>
+      <c r="J94" s="263" t="s">
         <v>569</v>
       </c>
-      <c r="K94" s="295"/>
-      <c r="L94" s="295" t="s">
+      <c r="K94" s="263"/>
+      <c r="L94" s="263" t="s">
         <v>570</v>
       </c>
-      <c r="M94" s="295"/>
+      <c r="M94" s="263"/>
       <c r="N94" s="239" t="s">
         <v>571</v>
       </c>
@@ -36491,43 +36491,43 @@
       <c r="AE95" s="227"/>
     </row>
     <row r="96" spans="2:31" ht="15" customHeight="1">
-      <c r="B96" s="319" t="s">
+      <c r="B96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="C96" s="319" t="s">
+      <c r="C96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="D96" s="319" t="s">
+      <c r="D96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="E96" s="319" t="s">
+      <c r="E96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="F96" s="319" t="s">
+      <c r="F96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="G96" s="319" t="s">
+      <c r="G96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="H96" s="319" t="s">
+      <c r="H96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="I96" s="319" t="s">
+      <c r="I96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="J96" s="319" t="s">
+      <c r="J96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="K96" s="319" t="s">
+      <c r="K96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="L96" s="319" t="s">
+      <c r="L96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="M96" s="319" t="s">
+      <c r="M96" s="264" t="s">
         <v>572</v>
       </c>
-      <c r="N96" s="319" t="s">
+      <c r="N96" s="264" t="s">
         <v>572</v>
       </c>
       <c r="O96" s="227"/>
@@ -36998,6 +36998,76 @@
     </row>
   </sheetData>
   <mergeCells count="80">
+    <mergeCell ref="B2:N3"/>
+    <mergeCell ref="B4:N4"/>
+    <mergeCell ref="B6:N6"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F18"/>
+    <mergeCell ref="B19:F21"/>
+    <mergeCell ref="B22:F24"/>
+    <mergeCell ref="B25:F27"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="G15:N15"/>
+    <mergeCell ref="G34:N34"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="L35:M35"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="L36:M36"/>
+    <mergeCell ref="G37:K37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="L38:M38"/>
+    <mergeCell ref="G39:K39"/>
+    <mergeCell ref="L39:M39"/>
+    <mergeCell ref="G40:K40"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="G41:K41"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="L45:M45"/>
+    <mergeCell ref="G46:K46"/>
+    <mergeCell ref="L46:M46"/>
+    <mergeCell ref="G47:K47"/>
+    <mergeCell ref="L47:M47"/>
+    <mergeCell ref="G48:K48"/>
+    <mergeCell ref="L48:M48"/>
+    <mergeCell ref="B50:N51"/>
+    <mergeCell ref="B52:N52"/>
+    <mergeCell ref="B54:G54"/>
+    <mergeCell ref="H54:N54"/>
+    <mergeCell ref="J55:K55"/>
+    <mergeCell ref="L55:M55"/>
+    <mergeCell ref="J56:K56"/>
+    <mergeCell ref="L56:M56"/>
+    <mergeCell ref="J57:K57"/>
+    <mergeCell ref="L57:M57"/>
+    <mergeCell ref="J58:K58"/>
+    <mergeCell ref="L58:M58"/>
+    <mergeCell ref="J59:K59"/>
+    <mergeCell ref="L59:M59"/>
+    <mergeCell ref="B61:G61"/>
+    <mergeCell ref="H61:N61"/>
+    <mergeCell ref="B78:H78"/>
+    <mergeCell ref="B79:H81"/>
+    <mergeCell ref="B82:H84"/>
+    <mergeCell ref="B85:H87"/>
+    <mergeCell ref="I78:N78"/>
+    <mergeCell ref="I79:N81"/>
+    <mergeCell ref="I82:N84"/>
+    <mergeCell ref="I85:N87"/>
+    <mergeCell ref="B89:N89"/>
+    <mergeCell ref="C90:I90"/>
+    <mergeCell ref="J90:K90"/>
+    <mergeCell ref="L90:M90"/>
+    <mergeCell ref="C91:I91"/>
+    <mergeCell ref="J91:K91"/>
+    <mergeCell ref="L91:M91"/>
     <mergeCell ref="C94:I94"/>
     <mergeCell ref="J94:K94"/>
     <mergeCell ref="L94:M94"/>
@@ -37008,76 +37078,6 @@
     <mergeCell ref="C93:I93"/>
     <mergeCell ref="J93:K93"/>
     <mergeCell ref="L93:M93"/>
-    <mergeCell ref="B89:N89"/>
-    <mergeCell ref="C90:I90"/>
-    <mergeCell ref="J90:K90"/>
-    <mergeCell ref="L90:M90"/>
-    <mergeCell ref="C91:I91"/>
-    <mergeCell ref="J91:K91"/>
-    <mergeCell ref="L91:M91"/>
-    <mergeCell ref="B79:H81"/>
-    <mergeCell ref="B82:H84"/>
-    <mergeCell ref="B85:H87"/>
-    <mergeCell ref="I78:N78"/>
-    <mergeCell ref="I79:N81"/>
-    <mergeCell ref="I82:N84"/>
-    <mergeCell ref="I85:N87"/>
-    <mergeCell ref="J59:K59"/>
-    <mergeCell ref="L59:M59"/>
-    <mergeCell ref="B61:G61"/>
-    <mergeCell ref="H61:N61"/>
-    <mergeCell ref="B78:H78"/>
-    <mergeCell ref="J56:K56"/>
-    <mergeCell ref="L56:M56"/>
-    <mergeCell ref="J57:K57"/>
-    <mergeCell ref="L57:M57"/>
-    <mergeCell ref="J58:K58"/>
-    <mergeCell ref="L58:M58"/>
-    <mergeCell ref="B50:N51"/>
-    <mergeCell ref="B52:N52"/>
-    <mergeCell ref="B54:G54"/>
-    <mergeCell ref="H54:N54"/>
-    <mergeCell ref="J55:K55"/>
-    <mergeCell ref="L55:M55"/>
-    <mergeCell ref="G46:K46"/>
-    <mergeCell ref="L46:M46"/>
-    <mergeCell ref="G47:K47"/>
-    <mergeCell ref="L47:M47"/>
-    <mergeCell ref="G48:K48"/>
-    <mergeCell ref="L48:M48"/>
-    <mergeCell ref="G43:K43"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="L44:M44"/>
-    <mergeCell ref="G45:K45"/>
-    <mergeCell ref="L45:M45"/>
-    <mergeCell ref="G40:K40"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="G41:K41"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="G42:K42"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="G37:K37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="G38:K38"/>
-    <mergeCell ref="L38:M38"/>
-    <mergeCell ref="G39:K39"/>
-    <mergeCell ref="L39:M39"/>
-    <mergeCell ref="G34:N34"/>
-    <mergeCell ref="G35:K35"/>
-    <mergeCell ref="L35:M35"/>
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="L36:M36"/>
-    <mergeCell ref="B19:F21"/>
-    <mergeCell ref="B22:F24"/>
-    <mergeCell ref="B25:F27"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="G15:N15"/>
-    <mergeCell ref="B2:N3"/>
-    <mergeCell ref="B4:N4"/>
-    <mergeCell ref="B6:N6"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F18"/>
   </mergeCells>
   <conditionalFormatting sqref="E9:E12">
     <cfRule type="cellIs" dxfId="7" priority="1" operator="lessThan">

</xml_diff>